<commit_message>
Actualiza el archivo de pruebas excel con los resultados del 3er sprint
</commit_message>
<xml_diff>
--- a/docs/Pruebas_Unitarias_CMQ_V4.xlsx
+++ b/docs/Pruebas_Unitarias_CMQ_V4.xlsx
@@ -5,28 +5,23 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\crist\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\crist\PROYECTOS_2026_I\Proyecto_IngSoft_SP4\PRUEBAS_UNITARIAS_SPRINT3-4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CCB78B6-12E8-4817-A039-BFC557DBCDB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25280CD7-B252-4ED9-86CE-145F235F8037}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sprint 3 - Citas Médicas" sheetId="1" r:id="rId1"/>
     <sheet name="Sprint 4 - Enfermería" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0" iterateDelta="1E-4"/>
-  <extLst>
-    <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
-      <loext:extCalcPr stringRefSyntax="ExcelA1"/>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="171">
   <si>
     <t>TABLA DE PRUEBAS UNITARIAS — MÓDULO SECRETARÍA / GESTIÓN DE CITAS MÉDICAS</t>
   </si>
@@ -302,9 +297,6 @@
     <t>En el modal de edición se cambia la fecha y hora de la cita a una fecha que ya pasó y se intenta guardar.</t>
   </si>
   <si>
-    <t>El modal permitía guardar fechas pasadas en la edición, reactivando citas ya vencidas o con fechas incorrectas.</t>
-  </si>
-  <si>
     <t>PU-CM-012</t>
   </si>
   <si>
@@ -314,9 +306,6 @@
     <t>En el modal de edición se modifican campos válidos (médico o fecha futura válida) y se presiona 'Guardar Cambios'.</t>
   </si>
   <si>
-    <t>Tras guardar exitosamente, el modal no se cerraba automáticamente y la tabla no se actualizaba, requiriendo recarga manual.</t>
-  </si>
-  <si>
     <t>PU-CM-013</t>
   </si>
   <si>
@@ -518,22 +507,117 @@
     <t>Se selecciona una fecha y hora anterior al momento actual (ej. ayer o hace una hora) en el campo datetime-local(ingresando hora manualmente).</t>
   </si>
   <si>
-    <t>CORREGIR, no funciona la propuesta de codigo</t>
-  </si>
-  <si>
-    <t>PENDIENTE</t>
-  </si>
-  <si>
-    <t>5/13.</t>
-  </si>
-  <si>
-    <t>0/15.</t>
-  </si>
-  <si>
-    <t>Total de casos probados: 15    |    Casos resueltos: 0    |    Casos pendientes: 15</t>
-  </si>
-  <si>
-    <t>Total de casos probados: 13    |    Casos resueltos: 5    |    Casos pendientes: 8</t>
+    <t>const citasFiltradas = citas.filter(c =&gt;
+  c.nombre.toLowerCase()
+    .includes(busqueda.toLowerCase()) ||
+  c.pacDocumento.includes(busqueda)
+)</t>
+  </si>
+  <si>
+    <t>La tabla debe filtrar y mostrar únicamente las citas del paciente buscado, sin distinción de mayúsculas/minúsculas.</t>
+  </si>
+  <si>
+    <t>La tabla se actualiza en tiempo real mostrando solo las citas que coinciden con el texto ingresado, sin distinción de caso.</t>
+  </si>
+  <si>
+    <t>{citasFiltradas.length === 0 &amp;&amp; (
+  &lt;tr&gt;
+    &lt;td colSpan='6' className='no-results'&gt;
+      No se encontraron citas
+    &lt;/td&gt;
+  &lt;/tr&gt;
+)}</t>
+  </si>
+  <si>
+    <t>La tabla debe mostrar el mensaje 'No se encontraron citas' centrado cuando ningún resultado coincide con la búsqueda.</t>
+  </si>
+  <si>
+    <t>La tabla muestra el mensaje 'No se encontraron citas' en la fila de resultados cuando la búsqueda no arroja coincidencias.</t>
+  </si>
+  <si>
+    <t>// El filtro opera sobre el estado 'busqueda'
+// Si busqueda === '' el filter retorna todos los elementos
+const citasFiltradas = citas.filter(c =&gt;
+  c.nombre.toLowerCase()
+    .includes(busqueda.toLowerCase()) ||
+  c.pacDocumento.includes(busqueda)
+)
+// Con busqueda vacío, includes('') siempre es true</t>
+  </si>
+  <si>
+    <t>Con el campo de búsqueda vacío, la tabla debe mostrar la totalidad de citas registradas en el sistema.</t>
+  </si>
+  <si>
+    <t>Al limpiar el campo de búsqueda la tabla restaura y muestra todas las citas registradas correctamente.</t>
+  </si>
+  <si>
+    <t>if (!citaEditando.fecha) {
+  errsM.fecha = 'Selecciona una fecha'
+} else if (citaEditando.fecha &lt; ahoraLocal) {
+  errsM.fecha = 'No se pueden ingresar fechas pasadas'
+} else {
+  const disp = validarDisponibilidad(
+    citaEditando.fecha, citaEditando.medId, citas)
+  if (!disp.disponible) errsM.fecha = disp.mensaje
+}</t>
+  </si>
+  <si>
+    <t>El modal debe mostrar 'No se pueden ingresar fechas pasadas' bajo el campo de fecha y bloquear el guardado.</t>
+  </si>
+  <si>
+    <t>El modal resalta el campo de fecha en rojo, muestra el mensaje de error y no realiza la petición PUT al servidor.</t>
+  </si>
+  <si>
+    <t>El modal se cierra, se muestra el toast de confirmación en verde y la tabla actualiza los datos de la cita sin recargar la página.</t>
+  </si>
+  <si>
+    <t>// Botón Cancelar:
+&lt;button className='btn-cancelar'
+  onClick={() =&gt; setCitaEditando(null)}&gt;
+  Cancelar
+&lt;/button&gt;
+// Overlay también cierra:
+&lt;div className='modal-overlay'
+  onClick={() =&gt; setCitaEditando(null)}&gt;</t>
+  </si>
+  <si>
+    <t>El modal debe cerrarse sin guardar ningún cambio y la cita debe permanecer con sus datos originales al reabrirse.</t>
+  </si>
+  <si>
+    <t>Al cancelar o hacer clic fuera, el modal se cierra y los datos originales de la cita permanecen intactos en la tabla.</t>
+  </si>
+  <si>
+    <t>13/13.</t>
+  </si>
+  <si>
+    <t>Total de casos probados: 13    |    Casos resueltos: 13   |    Casos pendientes: 0</t>
+  </si>
+  <si>
+    <t>El modal debe cerrarse automáticamente, mostrar el toast ' Cita modificada exitosamente' y reflejar los cambios en la tabla de citas.</t>
+  </si>
+  <si>
+    <t>if (data.success) {
+  await cargarDatos()
+  setCitaEditando(null)
+  setErroresModal({})
+  setExitoMsg(' Cita modificada exitosamente')
+  setTimeout(() =&gt; setExitoMsg(''), 4000)
+}</t>
+  </si>
+  <si>
+    <t>Tras guardar exitosamente, el modal no se cerraba automáticamente y la tabla no se actualizaba, requiriendo recarga manual y tampoco existia un respectivo mensaje de confirmacion.</t>
+  </si>
+  <si>
+    <t>El modal permitía guardar fechas pasadas en la edición(manualmente), reactivando citas ya vencidas o con fechas incorrectas.</t>
+  </si>
+  <si>
+    <t>(reingresar al modal de edicion)</t>
+  </si>
+  <si>
+    <t>Total de casos probados: 15    |    Casos resueltos: 15    |    Casos pendientes: 0</t>
+  </si>
+  <si>
+    <t>15/15.</t>
   </si>
 </sst>
 </file>
@@ -614,22 +698,21 @@
     </font>
     <font>
       <b/>
-      <sz val="9"/>
-      <color rgb="FF16A34A"/>
+      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="9"/>
-      <color rgb="FFFF0000"/>
+      <color rgb="FF00B050"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
     <font>
-      <b/>
       <sz val="10"/>
-      <color rgb="FFFFFFFF"/>
+      <color rgb="FF475569"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -717,17 +800,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -753,23 +827,61 @@
     <xf numFmtId="0" fontId="10" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1114,6 +1226,417 @@
         <a:xfrm>
           <a:off x="16411575" y="17102841"/>
           <a:ext cx="6659226" cy="566140"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>52871</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>403778</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>6087719</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>2024185</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="8" name="Imagen 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E5D32A70-1EC8-B376-927B-805075FA2872}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="16379963" y="19112120"/>
+          <a:ext cx="6034848" cy="1620407"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>52871</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>341658</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>5808181</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>2240249</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="9" name="Imagen 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F70C2589-CD1E-3620-AE1C-ED840B5F1E5A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="16379963" y="21586549"/>
+          <a:ext cx="5755310" cy="1898591"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>1191730</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>32221</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>4897093</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>3174</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="10" name="Imagen 9">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CB6A67E0-87C8-5299-54EF-1D61BE2BB5EA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="17518822" y="23813661"/>
+          <a:ext cx="3705363" cy="2500004"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>1626567</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>32525</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>4596849</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>2504404</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="11" name="Imagen 10">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{75364664-F912-9507-B981-96D332508D46}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="17953659" y="26350514"/>
+          <a:ext cx="2970282" cy="2471879"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>1335570</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>766142</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>5038542</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>1697935</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="12" name="Imagen 11">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2CF3E898-B3B0-1335-D1FE-3513F9B282B5}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="17662662" y="29620680"/>
+          <a:ext cx="3702972" cy="931793"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>331305</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>100025</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>2049946</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>2497806</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="13" name="Imagen 12">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5E720C27-4B2C-6008-9E70-902537A4915D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="16658397" y="31491112"/>
+          <a:ext cx="1718641" cy="2397781"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>2536550</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>1449456</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>3592582</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>1449456</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="15" name="Conector recto de flecha 14">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2BFA8468-1C62-237E-7F44-92577552DCF4}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="18863642" y="32840543"/>
+          <a:ext cx="1056032" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="dk1"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:round/>
+          <a:headEnd type="none" w="med" len="med"/>
+          <a:tailEnd type="arrow" w="med" len="med"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>4017063</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>122362</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>5756412</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>2524645</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="16" name="Imagen 15">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A16709CA-5EDB-EDEF-6F01-32E0CE0F8C9A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId13"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="20344155" y="31513449"/>
+          <a:ext cx="1739349" cy="2402283"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>72473</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>481104</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>6004892</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>1901098</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="17" name="Imagen 16">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3D92C5EA-82F9-F863-4703-B0CB1CE56096}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId14"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="16399565" y="14116349"/>
+          <a:ext cx="5932419" cy="1419994"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1304,6 +1827,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:J17"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1346,404 +1872,442 @@
       <c r="I2" s="14"/>
     </row>
     <row r="3" spans="1:10" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="F3" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="G3" s="4" t="s">
+      <c r="G3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="H3" s="4" t="s">
+      <c r="H3" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="I3" s="4" t="s">
+      <c r="I3" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="J3" s="4" t="s">
+      <c r="J3" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="200.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="5">
+      <c r="A4" s="2">
         <v>1</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="E4" s="7" t="s">
+      <c r="E4" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F4" s="8" t="s">
+      <c r="F4" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="G4" s="6" t="s">
+      <c r="G4" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="H4" s="6" t="s">
+      <c r="H4" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="I4" s="9" t="s">
+      <c r="I4" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="J4" s="10"/>
+      <c r="J4" s="7"/>
     </row>
     <row r="5" spans="1:10" ht="200.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="5">
+      <c r="A5" s="2">
         <v>2</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="E5" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="F5" s="8" t="s">
+      <c r="F5" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="G5" s="6" t="s">
+      <c r="G5" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="H5" s="6" t="s">
+      <c r="H5" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="I5" s="9" t="s">
+      <c r="I5" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="J5" s="10"/>
+      <c r="J5" s="7"/>
     </row>
     <row r="6" spans="1:10" ht="200.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="5">
+      <c r="A6" s="2">
         <v>3</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D6" s="11" t="s">
+      <c r="D6" s="8" t="s">
+        <v>145</v>
+      </c>
+      <c r="E6" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="I6" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="J6" s="7"/>
+    </row>
+    <row r="7" spans="1:10" ht="200.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="2">
+        <v>4</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="I7" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="J7" s="7"/>
+    </row>
+    <row r="8" spans="1:10" ht="200.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="2">
+        <v>5</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="I8" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="J8" s="7"/>
+    </row>
+    <row r="9" spans="1:10" ht="200.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="2">
+        <v>6</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="H9" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="I9" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="J9" s="7"/>
+    </row>
+    <row r="10" spans="1:10" ht="200.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="2">
+        <v>7</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="I10" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="J10" s="7"/>
+    </row>
+    <row r="11" spans="1:10" ht="200.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="2">
+        <v>8</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="F11" s="16" t="s">
+        <v>146</v>
+      </c>
+      <c r="G11" s="15" t="s">
         <v>147</v>
       </c>
-      <c r="E6" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="F6" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="G6" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="H6" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="I6" s="9" t="s">
+      <c r="H11" s="15" t="s">
+        <v>148</v>
+      </c>
+      <c r="I11" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="J6" s="10"/>
-    </row>
-    <row r="7" spans="1:10" ht="200.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="5">
-        <v>4</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="E7" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="F7" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="G7" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="H7" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="I7" s="9" t="s">
+      <c r="J11" s="7"/>
+    </row>
+    <row r="12" spans="1:10" ht="200.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="2">
+        <v>9</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="F12" s="16" t="s">
+        <v>149</v>
+      </c>
+      <c r="G12" s="15" t="s">
+        <v>150</v>
+      </c>
+      <c r="H12" s="15" t="s">
+        <v>151</v>
+      </c>
+      <c r="I12" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="J7" s="10"/>
-    </row>
-    <row r="8" spans="1:10" ht="200.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="5">
-        <v>5</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="D8" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="E8" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="F8" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="G8" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="H8" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="I8" s="9" t="s">
+      <c r="J12" s="7"/>
+    </row>
+    <row r="13" spans="1:10" ht="200.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="2">
+        <v>10</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="F13" s="16" t="s">
+        <v>152</v>
+      </c>
+      <c r="G13" s="15" t="s">
+        <v>153</v>
+      </c>
+      <c r="H13" s="15" t="s">
+        <v>154</v>
+      </c>
+      <c r="I13" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="J8" s="10"/>
-    </row>
-    <row r="9" spans="1:10" ht="200.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="5">
-        <v>6</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="D9" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="E9" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="F9" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="G9" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="H9" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="I9" s="16" t="s">
-        <v>148</v>
-      </c>
-      <c r="J9" s="10"/>
-    </row>
-    <row r="10" spans="1:10" ht="200.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="5">
-        <v>7</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="C10" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="D10" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="E10" s="7" t="s">
-        <v>57</v>
-      </c>
-      <c r="F10" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="G10" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="H10" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="I10" s="9" t="s">
+      <c r="J13" s="7"/>
+    </row>
+    <row r="14" spans="1:10" ht="200.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="2">
+        <v>11</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="F14" s="16" t="s">
+        <v>155</v>
+      </c>
+      <c r="G14" s="15" t="s">
+        <v>156</v>
+      </c>
+      <c r="H14" s="15" t="s">
+        <v>157</v>
+      </c>
+      <c r="I14" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="J10" s="10"/>
-    </row>
-    <row r="11" spans="1:10" ht="200.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="5">
-        <v>8</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="C11" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="D11" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="E11" s="7" t="s">
-        <v>64</v>
-      </c>
-      <c r="F11" s="8"/>
-      <c r="G11" s="6"/>
-      <c r="H11" s="6"/>
-      <c r="I11" s="15" t="s">
-        <v>149</v>
-      </c>
-      <c r="J11" s="10"/>
-    </row>
-    <row r="12" spans="1:10" ht="200.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="5">
-        <v>9</v>
-      </c>
-      <c r="B12" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="C12" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="D12" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="E12" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="F12" s="8"/>
-      <c r="G12" s="6"/>
-      <c r="H12" s="6"/>
-      <c r="I12" s="15" t="s">
-        <v>149</v>
-      </c>
-      <c r="J12" s="10"/>
-    </row>
-    <row r="13" spans="1:10" ht="200.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="5">
-        <v>10</v>
-      </c>
-      <c r="B13" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="C13" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="D13" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="E13" s="7" t="s">
-        <v>72</v>
-      </c>
-      <c r="F13" s="8"/>
-      <c r="G13" s="6"/>
-      <c r="H13" s="6"/>
-      <c r="I13" s="15" t="s">
-        <v>149</v>
-      </c>
-      <c r="J13" s="10"/>
-    </row>
-    <row r="14" spans="1:10" ht="200.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="5">
-        <v>11</v>
-      </c>
-      <c r="B14" s="6" t="s">
-        <v>73</v>
-      </c>
-      <c r="C14" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="D14" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="E14" s="7" t="s">
+      <c r="J14" s="7"/>
+    </row>
+    <row r="15" spans="1:10" ht="200.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="2">
+        <v>12</v>
+      </c>
+      <c r="B15" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="F14" s="8"/>
-      <c r="G14" s="6"/>
-      <c r="H14" s="6"/>
-      <c r="I14" s="15" t="s">
-        <v>149</v>
-      </c>
-      <c r="J14" s="10"/>
-    </row>
-    <row r="15" spans="1:10" ht="200.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="5">
-        <v>12</v>
-      </c>
-      <c r="B15" s="6" t="s">
+      <c r="C15" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="C15" s="6" t="s">
+      <c r="D15" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="D15" s="6" t="s">
+      <c r="E15" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="F15" s="16" t="s">
+        <v>165</v>
+      </c>
+      <c r="G15" s="15" t="s">
+        <v>164</v>
+      </c>
+      <c r="H15" s="15" t="s">
+        <v>158</v>
+      </c>
+      <c r="I15" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J15" s="7"/>
+    </row>
+    <row r="16" spans="1:10" ht="200.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="2">
+        <v>13</v>
+      </c>
+      <c r="B16" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="E15" s="7" t="s">
+      <c r="C16" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="F15" s="8"/>
-      <c r="G15" s="6"/>
-      <c r="H15" s="6"/>
-      <c r="I15" s="15" t="s">
-        <v>149</v>
-      </c>
-      <c r="J15" s="10"/>
-    </row>
-    <row r="16" spans="1:10" ht="200.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="5">
-        <v>13</v>
-      </c>
-      <c r="B16" s="6" t="s">
+      <c r="D16" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="C16" s="6" t="s">
+      <c r="E16" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="D16" s="6" t="s">
-        <v>83</v>
-      </c>
-      <c r="E16" s="7" t="s">
-        <v>84</v>
-      </c>
-      <c r="F16" s="8"/>
-      <c r="G16" s="6"/>
-      <c r="H16" s="6"/>
-      <c r="I16" s="15" t="s">
-        <v>149</v>
-      </c>
-      <c r="J16" s="10"/>
+      <c r="F16" s="16" t="s">
+        <v>159</v>
+      </c>
+      <c r="G16" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="H16" s="15" t="s">
+        <v>161</v>
+      </c>
+      <c r="I16" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J16" s="18" t="s">
+        <v>168</v>
+      </c>
     </row>
     <row r="17" spans="1:9" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="18" t="s">
-        <v>153</v>
-      </c>
-      <c r="B17" s="1"/>
-      <c r="C17" s="1"/>
-      <c r="D17" s="1"/>
-      <c r="E17" s="1"/>
-      <c r="F17" s="1"/>
-      <c r="G17" s="1"/>
-      <c r="H17" s="1"/>
-      <c r="I17" s="17" t="s">
-        <v>150</v>
+      <c r="A17" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="B17" s="12"/>
+      <c r="C17" s="12"/>
+      <c r="D17" s="12"/>
+      <c r="E17" s="12"/>
+      <c r="F17" s="12"/>
+      <c r="G17" s="12"/>
+      <c r="H17" s="12"/>
+      <c r="I17" s="10" t="s">
+        <v>162</v>
       </c>
     </row>
   </sheetData>
@@ -1753,8 +2317,8 @@
     <mergeCell ref="A17:H17"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
-  <drawing r:id="rId1"/>
+  <pageSetup paperSize="9" scale="24" fitToHeight="0" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -1776,437 +2340,438 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="13" t="s">
+        <v>83</v>
+      </c>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="13"/>
+      <c r="I1" s="13"/>
+    </row>
+    <row r="2" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="20" t="s">
+        <v>84</v>
+      </c>
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
+      <c r="H2" s="14"/>
+      <c r="I2" s="14"/>
+    </row>
+    <row r="3" spans="1:10" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="22" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="22" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3" s="22" t="s">
+        <v>4</v>
+      </c>
+      <c r="D3" s="22" t="s">
+        <v>5</v>
+      </c>
+      <c r="E3" s="22" t="s">
+        <v>6</v>
+      </c>
+      <c r="F3" s="22" t="s">
+        <v>7</v>
+      </c>
+      <c r="G3" s="22" t="s">
+        <v>8</v>
+      </c>
+      <c r="H3" s="22" t="s">
+        <v>9</v>
+      </c>
+      <c r="I3" s="22" t="s">
+        <v>10</v>
+      </c>
+      <c r="J3" s="22" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="200.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="23">
+        <v>1</v>
+      </c>
+      <c r="B4" s="24" t="s">
         <v>85</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
-      <c r="H1" s="3"/>
-      <c r="I1" s="3"/>
-    </row>
-    <row r="2" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+      <c r="C4" s="24" t="s">
         <v>86</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
-    </row>
-    <row r="3" spans="1:10" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
+      <c r="D4" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="E4" s="25" t="s">
+        <v>88</v>
+      </c>
+      <c r="F4" s="26"/>
+      <c r="G4" s="24"/>
+      <c r="H4" s="24"/>
+      <c r="I4" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="J4" s="28"/>
+    </row>
+    <row r="5" spans="1:10" ht="200.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="23">
         <v>2</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B5" s="24" t="s">
+        <v>89</v>
+      </c>
+      <c r="C5" s="24" t="s">
+        <v>90</v>
+      </c>
+      <c r="D5" s="24" t="s">
+        <v>91</v>
+      </c>
+      <c r="E5" s="25" t="s">
+        <v>92</v>
+      </c>
+      <c r="F5" s="26"/>
+      <c r="G5" s="24"/>
+      <c r="H5" s="24"/>
+      <c r="I5" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="J5" s="28"/>
+    </row>
+    <row r="6" spans="1:10" ht="200.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="23">
         <v>3</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="B6" s="24" t="s">
+        <v>93</v>
+      </c>
+      <c r="C6" s="24" t="s">
+        <v>94</v>
+      </c>
+      <c r="D6" s="24" t="s">
+        <v>95</v>
+      </c>
+      <c r="E6" s="25" t="s">
+        <v>96</v>
+      </c>
+      <c r="F6" s="26"/>
+      <c r="G6" s="24"/>
+      <c r="H6" s="24"/>
+      <c r="I6" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="J6" s="28"/>
+    </row>
+    <row r="7" spans="1:10" ht="200.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="23">
         <v>4</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="B7" s="24" t="s">
+        <v>97</v>
+      </c>
+      <c r="C7" s="24" t="s">
+        <v>98</v>
+      </c>
+      <c r="D7" s="24" t="s">
+        <v>99</v>
+      </c>
+      <c r="E7" s="25" t="s">
+        <v>100</v>
+      </c>
+      <c r="F7" s="26"/>
+      <c r="G7" s="24"/>
+      <c r="H7" s="24"/>
+      <c r="I7" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="J7" s="28"/>
+    </row>
+    <row r="8" spans="1:10" ht="200.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="23">
         <v>5</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="B8" s="24" t="s">
+        <v>101</v>
+      </c>
+      <c r="C8" s="24" t="s">
+        <v>102</v>
+      </c>
+      <c r="D8" s="24" t="s">
+        <v>103</v>
+      </c>
+      <c r="E8" s="25" t="s">
+        <v>104</v>
+      </c>
+      <c r="F8" s="26"/>
+      <c r="G8" s="24"/>
+      <c r="H8" s="24"/>
+      <c r="I8" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="J8" s="28"/>
+    </row>
+    <row r="9" spans="1:10" ht="200.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="23">
         <v>6</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="B9" s="24" t="s">
+        <v>105</v>
+      </c>
+      <c r="C9" s="24" t="s">
+        <v>106</v>
+      </c>
+      <c r="D9" s="24" t="s">
+        <v>107</v>
+      </c>
+      <c r="E9" s="25" t="s">
+        <v>108</v>
+      </c>
+      <c r="F9" s="26"/>
+      <c r="G9" s="24"/>
+      <c r="H9" s="24"/>
+      <c r="I9" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="J9" s="28"/>
+    </row>
+    <row r="10" spans="1:10" ht="200.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="23">
         <v>7</v>
       </c>
-      <c r="G3" s="4" t="s">
+      <c r="B10" s="24" t="s">
+        <v>109</v>
+      </c>
+      <c r="C10" s="24" t="s">
+        <v>110</v>
+      </c>
+      <c r="D10" s="24" t="s">
+        <v>111</v>
+      </c>
+      <c r="E10" s="25" t="s">
+        <v>112</v>
+      </c>
+      <c r="F10" s="26"/>
+      <c r="G10" s="24"/>
+      <c r="H10" s="24"/>
+      <c r="I10" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="J10" s="28"/>
+    </row>
+    <row r="11" spans="1:10" ht="200.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="23">
         <v>8</v>
       </c>
-      <c r="H3" s="4" t="s">
+      <c r="B11" s="24" t="s">
+        <v>113</v>
+      </c>
+      <c r="C11" s="24" t="s">
+        <v>114</v>
+      </c>
+      <c r="D11" s="24" t="s">
+        <v>115</v>
+      </c>
+      <c r="E11" s="25" t="s">
+        <v>116</v>
+      </c>
+      <c r="F11" s="26"/>
+      <c r="G11" s="24"/>
+      <c r="H11" s="24"/>
+      <c r="I11" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="J11" s="28"/>
+    </row>
+    <row r="12" spans="1:10" ht="200.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="23">
         <v>9</v>
       </c>
-      <c r="I3" s="4" t="s">
+      <c r="B12" s="24" t="s">
+        <v>117</v>
+      </c>
+      <c r="C12" s="24" t="s">
+        <v>118</v>
+      </c>
+      <c r="D12" s="24" t="s">
+        <v>119</v>
+      </c>
+      <c r="E12" s="25" t="s">
+        <v>120</v>
+      </c>
+      <c r="F12" s="26"/>
+      <c r="G12" s="24"/>
+      <c r="H12" s="24"/>
+      <c r="I12" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="J12" s="28"/>
+    </row>
+    <row r="13" spans="1:10" ht="200.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="23">
         <v>10</v>
       </c>
-      <c r="J3" s="4" t="s">
+      <c r="B13" s="24" t="s">
+        <v>121</v>
+      </c>
+      <c r="C13" s="24" t="s">
+        <v>122</v>
+      </c>
+      <c r="D13" s="24" t="s">
+        <v>123</v>
+      </c>
+      <c r="E13" s="25" t="s">
+        <v>124</v>
+      </c>
+      <c r="F13" s="26"/>
+      <c r="G13" s="24"/>
+      <c r="H13" s="24"/>
+      <c r="I13" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="J13" s="28"/>
+    </row>
+    <row r="14" spans="1:10" ht="200.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="23">
         <v>11</v>
       </c>
-    </row>
-    <row r="4" spans="1:10" ht="109.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="5">
-        <v>1</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="D4" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="E4" s="7" t="s">
-        <v>90</v>
-      </c>
-      <c r="F4" s="8"/>
-      <c r="G4" s="6"/>
-      <c r="H4" s="6"/>
-      <c r="I4" s="9" t="s">
-        <v>149</v>
-      </c>
-      <c r="J4" s="10"/>
-    </row>
-    <row r="5" spans="1:10" ht="109.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="5">
-        <v>2</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>91</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>93</v>
-      </c>
-      <c r="E5" s="7" t="s">
-        <v>94</v>
-      </c>
-      <c r="F5" s="8"/>
-      <c r="G5" s="6"/>
-      <c r="H5" s="6"/>
-      <c r="I5" s="9" t="s">
-        <v>149</v>
-      </c>
-      <c r="J5" s="10"/>
-    </row>
-    <row r="6" spans="1:10" ht="109.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="5">
-        <v>3</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>95</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>96</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>97</v>
-      </c>
-      <c r="E6" s="7" t="s">
-        <v>98</v>
-      </c>
-      <c r="F6" s="8"/>
-      <c r="G6" s="6"/>
-      <c r="H6" s="6"/>
-      <c r="I6" s="9" t="s">
-        <v>149</v>
-      </c>
-      <c r="J6" s="10"/>
-    </row>
-    <row r="7" spans="1:10" ht="109.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="5">
-        <v>4</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>101</v>
-      </c>
-      <c r="E7" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="F7" s="8"/>
-      <c r="G7" s="6"/>
-      <c r="H7" s="6"/>
-      <c r="I7" s="9" t="s">
-        <v>149</v>
-      </c>
-      <c r="J7" s="10"/>
-    </row>
-    <row r="8" spans="1:10" ht="109.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="5">
-        <v>5</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>103</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>104</v>
-      </c>
-      <c r="D8" s="6" t="s">
-        <v>105</v>
-      </c>
-      <c r="E8" s="7" t="s">
-        <v>106</v>
-      </c>
-      <c r="F8" s="8"/>
-      <c r="G8" s="6"/>
-      <c r="H8" s="6"/>
-      <c r="I8" s="9" t="s">
-        <v>149</v>
-      </c>
-      <c r="J8" s="10"/>
-    </row>
-    <row r="9" spans="1:10" ht="109.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="5">
-        <v>6</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>107</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>108</v>
-      </c>
-      <c r="D9" s="6" t="s">
-        <v>109</v>
-      </c>
-      <c r="E9" s="7" t="s">
-        <v>110</v>
-      </c>
-      <c r="F9" s="8"/>
-      <c r="G9" s="6"/>
-      <c r="H9" s="6"/>
-      <c r="I9" s="9" t="s">
-        <v>149</v>
-      </c>
-      <c r="J9" s="10"/>
-    </row>
-    <row r="10" spans="1:10" ht="109.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="5">
-        <v>7</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>111</v>
-      </c>
-      <c r="C10" s="6" t="s">
-        <v>112</v>
-      </c>
-      <c r="D10" s="6" t="s">
-        <v>113</v>
-      </c>
-      <c r="E10" s="7" t="s">
-        <v>114</v>
-      </c>
-      <c r="F10" s="8"/>
-      <c r="G10" s="6"/>
-      <c r="H10" s="6"/>
-      <c r="I10" s="9" t="s">
-        <v>149</v>
-      </c>
-      <c r="J10" s="10"/>
-    </row>
-    <row r="11" spans="1:10" ht="109.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="5">
-        <v>8</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>115</v>
-      </c>
-      <c r="C11" s="6" t="s">
-        <v>116</v>
-      </c>
-      <c r="D11" s="6" t="s">
-        <v>117</v>
-      </c>
-      <c r="E11" s="7" t="s">
-        <v>118</v>
-      </c>
-      <c r="F11" s="8"/>
-      <c r="G11" s="6"/>
-      <c r="H11" s="6"/>
-      <c r="I11" s="9" t="s">
-        <v>149</v>
-      </c>
-      <c r="J11" s="10"/>
-    </row>
-    <row r="12" spans="1:10" ht="109.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="5">
-        <v>9</v>
-      </c>
-      <c r="B12" s="6" t="s">
-        <v>119</v>
-      </c>
-      <c r="C12" s="6" t="s">
-        <v>120</v>
-      </c>
-      <c r="D12" s="6" t="s">
-        <v>121</v>
-      </c>
-      <c r="E12" s="7" t="s">
-        <v>122</v>
-      </c>
-      <c r="F12" s="8"/>
-      <c r="G12" s="6"/>
-      <c r="H12" s="6"/>
-      <c r="I12" s="9" t="s">
-        <v>149</v>
-      </c>
-      <c r="J12" s="10"/>
-    </row>
-    <row r="13" spans="1:10" ht="109.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="5">
-        <v>10</v>
-      </c>
-      <c r="B13" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="C13" s="6" t="s">
-        <v>124</v>
-      </c>
-      <c r="D13" s="6" t="s">
+      <c r="B14" s="24" t="s">
         <v>125</v>
       </c>
-      <c r="E13" s="7" t="s">
+      <c r="C14" s="24" t="s">
         <v>126</v>
       </c>
-      <c r="F13" s="8"/>
-      <c r="G13" s="6"/>
-      <c r="H13" s="6"/>
-      <c r="I13" s="9" t="s">
-        <v>149</v>
-      </c>
-      <c r="J13" s="10"/>
-    </row>
-    <row r="14" spans="1:10" ht="109.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="5">
-        <v>11</v>
-      </c>
-      <c r="B14" s="6" t="s">
+      <c r="D14" s="24" t="s">
         <v>127</v>
       </c>
-      <c r="C14" s="6" t="s">
+      <c r="E14" s="25" t="s">
         <v>128</v>
       </c>
-      <c r="D14" s="6" t="s">
+      <c r="F14" s="26"/>
+      <c r="G14" s="24"/>
+      <c r="H14" s="24"/>
+      <c r="I14" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="J14" s="28"/>
+    </row>
+    <row r="15" spans="1:10" ht="200.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="23">
+        <v>12</v>
+      </c>
+      <c r="B15" s="24" t="s">
         <v>129</v>
       </c>
-      <c r="E14" s="7" t="s">
+      <c r="C15" s="24" t="s">
         <v>130</v>
       </c>
-      <c r="F14" s="8"/>
-      <c r="G14" s="6"/>
-      <c r="H14" s="6"/>
-      <c r="I14" s="9" t="s">
-        <v>149</v>
-      </c>
-      <c r="J14" s="10"/>
-    </row>
-    <row r="15" spans="1:10" ht="109.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="5">
-        <v>12</v>
-      </c>
-      <c r="B15" s="6" t="s">
+      <c r="D15" s="24" t="s">
         <v>131</v>
       </c>
-      <c r="C15" s="6" t="s">
+      <c r="E15" s="25" t="s">
         <v>132</v>
       </c>
-      <c r="D15" s="6" t="s">
+      <c r="F15" s="26"/>
+      <c r="G15" s="24"/>
+      <c r="H15" s="24"/>
+      <c r="I15" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="J15" s="28"/>
+    </row>
+    <row r="16" spans="1:10" ht="200.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="23">
+        <v>13</v>
+      </c>
+      <c r="B16" s="24" t="s">
         <v>133</v>
       </c>
-      <c r="E15" s="7" t="s">
+      <c r="C16" s="24" t="s">
         <v>134</v>
       </c>
-      <c r="F15" s="8"/>
-      <c r="G15" s="6"/>
-      <c r="H15" s="6"/>
-      <c r="I15" s="9" t="s">
-        <v>149</v>
-      </c>
-      <c r="J15" s="10"/>
-    </row>
-    <row r="16" spans="1:10" ht="109.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="5">
-        <v>13</v>
-      </c>
-      <c r="B16" s="6" t="s">
+      <c r="D16" s="24" t="s">
         <v>135</v>
       </c>
-      <c r="C16" s="6" t="s">
+      <c r="E16" s="25" t="s">
         <v>136</v>
       </c>
-      <c r="D16" s="6" t="s">
+      <c r="F16" s="26"/>
+      <c r="G16" s="24"/>
+      <c r="H16" s="24"/>
+      <c r="I16" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="J16" s="28"/>
+    </row>
+    <row r="17" spans="1:10" ht="200.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="23">
+        <v>14</v>
+      </c>
+      <c r="B17" s="24" t="s">
         <v>137</v>
       </c>
-      <c r="E16" s="7" t="s">
+      <c r="C17" s="24" t="s">
         <v>138</v>
       </c>
-      <c r="F16" s="8"/>
-      <c r="G16" s="6"/>
-      <c r="H16" s="6"/>
-      <c r="I16" s="9" t="s">
-        <v>149</v>
-      </c>
-      <c r="J16" s="10"/>
-    </row>
-    <row r="17" spans="1:10" ht="109.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="5">
-        <v>14</v>
-      </c>
-      <c r="B17" s="6" t="s">
+      <c r="D17" s="24" t="s">
         <v>139</v>
       </c>
-      <c r="C17" s="6" t="s">
+      <c r="E17" s="25" t="s">
         <v>140</v>
       </c>
-      <c r="D17" s="6" t="s">
+      <c r="F17" s="26"/>
+      <c r="G17" s="24"/>
+      <c r="H17" s="24"/>
+      <c r="I17" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="J17" s="28"/>
+    </row>
+    <row r="18" spans="1:10" ht="200.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="23">
+        <v>15</v>
+      </c>
+      <c r="B18" s="24" t="s">
         <v>141</v>
       </c>
-      <c r="E17" s="7" t="s">
+      <c r="C18" s="24" t="s">
         <v>142</v>
       </c>
-      <c r="F17" s="8"/>
-      <c r="G17" s="6"/>
-      <c r="H17" s="6"/>
-      <c r="I17" s="9" t="s">
-        <v>149</v>
-      </c>
-      <c r="J17" s="10"/>
-    </row>
-    <row r="18" spans="1:10" ht="109.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="5">
-        <v>15</v>
-      </c>
-      <c r="B18" s="6" t="s">
+      <c r="D18" s="24" t="s">
         <v>143</v>
       </c>
-      <c r="C18" s="6" t="s">
+      <c r="E18" s="25" t="s">
         <v>144</v>
       </c>
-      <c r="D18" s="6" t="s">
-        <v>145</v>
-      </c>
-      <c r="E18" s="7" t="s">
-        <v>146</v>
-      </c>
-      <c r="F18" s="8"/>
-      <c r="G18" s="6"/>
-      <c r="H18" s="6"/>
-      <c r="I18" s="9" t="s">
-        <v>149</v>
-      </c>
-      <c r="J18" s="10"/>
+      <c r="F18" s="26"/>
+      <c r="G18" s="24"/>
+      <c r="H18" s="24"/>
+      <c r="I18" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="J18" s="28"/>
     </row>
     <row r="19" spans="1:10" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="18" t="s">
-        <v>152</v>
-      </c>
-      <c r="B19" s="1"/>
-      <c r="C19" s="1"/>
-      <c r="D19" s="1"/>
-      <c r="E19" s="1"/>
-      <c r="F19" s="1"/>
-      <c r="G19" s="1"/>
-      <c r="H19" s="1"/>
-      <c r="I19" s="17" t="s">
-        <v>151</v>
-      </c>
+      <c r="A19" s="12" t="s">
+        <v>169</v>
+      </c>
+      <c r="B19" s="12"/>
+      <c r="C19" s="12"/>
+      <c r="D19" s="12"/>
+      <c r="E19" s="12"/>
+      <c r="F19" s="12"/>
+      <c r="G19" s="12"/>
+      <c r="H19" s="12"/>
+      <c r="I19" s="29" t="s">
+        <v>170</v>
+      </c>
+      <c r="J19" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>

<commit_message>
Actualiza el archivo de pruebas excel con los resultados del 4to Sprint
</commit_message>
<xml_diff>
--- a/docs/Pruebas_Unitarias_CMQ_V4.xlsx
+++ b/docs/Pruebas_Unitarias_CMQ_V4.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\crist\PROYECTOS_2026_I\Proyecto_IngSoft_SP4\PRUEBAS_UNITARIAS_SPRINT3-4\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\crist\PROYECTOS_2026_I\Proyecto_IngSoft_SP4\ultima_entrega_cmq\cmq-medical-data-integration\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25280CD7-B252-4ED9-86CE-145F235F8037}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8299BE4A-0B45-4185-85B4-C3076445E51A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sprint 3 - Citas Médicas" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="195">
   <si>
     <t>TABLA DE PRUEBAS UNITARIAS — MÓDULO SECRETARÍA / GESTIÓN DE CITAS MÉDICAS</t>
   </si>
@@ -468,42 +468,6 @@
     <t>El documento imprimible no tenía encabezado institucional ni mostraba el nombre del enfermero en turno, produciendo reportes sin autoría ni identificación.</t>
   </si>
   <si>
-    <t>PU-ENF-013</t>
-  </si>
-  <si>
-    <t>Registro PNI Secretaría / Teléfono con formato incorrecto</t>
-  </si>
-  <si>
-    <t>En el modal de registro de paciente PNI (emer.jsx), se ingresa un teléfono con menos o más de 10 dígitos o con letras (ej. '311abc', '123').</t>
-  </si>
-  <si>
-    <t>El modal de registro PNI no validaba el teléfono, permitiendo guardar números inválidos en la BD del paciente recién creado.</t>
-  </si>
-  <si>
-    <t>PU-ENF-014</t>
-  </si>
-  <si>
-    <t>Registro PNI Secretaría / Fecha de nacimiento futura</t>
-  </si>
-  <si>
-    <t>En el modal de registro PNI se selecciona una fecha de nacimiento posterior a la fecha actual (ej. un año en el futuro).</t>
-  </si>
-  <si>
-    <t>El modal de registro PNI aceptaba fechas de nacimiento futuras, generando edades negativas e inconsistencias en el historial del paciente.</t>
-  </si>
-  <si>
-    <t>PU-ENF-015</t>
-  </si>
-  <si>
-    <t>Registro PNI Secretaría / Ciudad con caracteres inválidos</t>
-  </si>
-  <si>
-    <t>En el modal de registro PNI se ingresa un nombre de ciudad con números o símbolos (ej. 'Bogot4', 'Call!', '123').</t>
-  </si>
-  <si>
-    <t>El sistema aceptaba nombres de ciudad con dígitos y símbolos especiales al registrar pacientes PNI, guardando datos no válidos.</t>
-  </si>
-  <si>
     <t>Se selecciona una fecha y hora anterior al momento actual (ej. ayer o hace una hora) en el campo datetime-local(ingresando hora manualmente).</t>
   </si>
   <si>
@@ -614,10 +578,219 @@
     <t>(reingresar al modal de edicion)</t>
   </si>
   <si>
-    <t>Total de casos probados: 15    |    Casos resueltos: 15    |    Casos pendientes: 0</t>
-  </si>
-  <si>
-    <t>15/15.</t>
+    <t>12/12.</t>
+  </si>
+  <si>
+    <t>Total de casos probados: 12    |    Casos resueltos: 12    |    Casos pendientes: 0</t>
+  </si>
+  <si>
+    <t>const errs = {}
+if (!formData.sintomas.trim())
+  errs.sintomas = 'Los síntomas son obligatorios'
+if (!formData.triage)
+  errs.triage = 'Seleccione un nivel de triage'
+if (!formData.presionArterial)
+  errs.presionArterial = 'La presión arterial es obligatoria'
+if (!formData.frecuenciaCardiaca)
+  errs.frecuenciaCardiaca = 'La frecuencia cardíaca es obligatoria'
+// ídem temperatura y saturación
+setErrors(errs)
+return Object.keys(errs).length === 0</t>
+  </si>
+  <si>
+    <t>El sistema debe resaltar en rojo cada campo faltante, mostrar el mensaje de error debajo de cada uno y bloquear el envío.</t>
+  </si>
+  <si>
+    <t>El sistema resalta los campos vacíos en rojo, muestra los mensajes de error debajo y no realiza la petición POST al API.</t>
+  </si>
+  <si>
+    <t>if (!formData.presionArterial) {
+  errs.presionArterial = 'La presión arterial es obligatoria'
+} else if (!/^\d{2,3}\/\d{2,3}$/.test(
+    formData.presionArterial)) {
+  errs.presionArterial = 'Formato inválido (Ej: 120/80)'
+}</t>
+  </si>
+  <si>
+    <t>El sistema debe mostrar 'Formato inválido (Ej: 120/80)' bajo el campo y bloquear el registro hasta ingresar el formato correcto.</t>
+  </si>
+  <si>
+    <t>El campo muestra borde rojo y el mensaje de validación del formato, impidiendo el guardado hasta corregir la presión arterial.</t>
+  </si>
+  <si>
+    <t>// Frecuencia cardíaca
+const fc = Number(formData.frecuenciaCardiaca)
+if (fc &lt; 20 || fc &gt; 250)
+  errs.frecuenciaCardiaca = 'Frecuencia inválida (rango: 20 – 250 LPM)'
+// Temperatura
+const t = Number(formData.temperatura)
+if (t &lt; 25 || t &gt; 45)
+  errs.temperatura = 'Temperatura inválida (rango: 25°C – 45°C)'
+// Saturación
+const sat = Number(formData.saturacion)
+if (sat &lt; 50 || sat &gt; 100)
+  errs.saturacion = 'Saturación inválida (rango: 50% – 100%)'</t>
+  </si>
+  <si>
+    <t>El sistema debe mostrar el mensaje de rango inválido bajo cada campo con valor fuera de límites y bloquear el guardado del triage.</t>
+  </si>
+  <si>
+    <t>El sistema muestra el mensaje de error de rango bajo cada campo infractor, resalta el campo en rojo y bloquea el envío del formulario.</t>
+  </si>
+  <si>
+    <t>const alertasSignos = () =&gt; {
+  const alertas = []
+  if (Number(formData.temperatura) &gt;= 38.5)
+    alertas.push('⚠️ Fiebre alta (≥38.5°C)')
+  if (Number(formData.saturacion) &lt; 90)
+    alertas.push('🔴 Saturación crítica (&lt;90%)')
+  if (Number(formData.frecuenciaCardiaca) &gt; 100)
+    alertas.push('⚠️ Taquicardia (&gt;100 LPM)')
+  if (Number(formData.frecuenciaCardiaca) &lt; 60)
+    alertas.push('⚠️ Bradicardia (&lt;60 LPM)')
+  return alertas
+}</t>
+  </si>
+  <si>
+    <t>El sistema debe mostrar un banner de alerta rojo con el mensaje correspondiente al umbral superado, sin bloquear el guardado.</t>
+  </si>
+  <si>
+    <t>El formulario muestra el banner de alertas clínicas con los mensajes de taquicardia, fiebre o saturación crítica en tiempo real al escribir.</t>
+  </si>
+  <si>
+    <t>if (!data.encontrado) {
+  setNoEncontrado(true)
+}
+// En el render se muestra el panel
+// 'Registrar como Urgencia' con campos:
+// urgNombre, urgGenero, urgTipoSangre
+// y el botón:
+// '🚨 Registrar como Urgencia y Continuar'</t>
+  </si>
+  <si>
+    <t>El sistema debe informar que el paciente no fue encontrado y mostrar un formulario para registrarlo como urgencia antes de continuar con el triage.</t>
+  </si>
+  <si>
+    <t>El sistema muestra el panel naranja de 'Registrar como Urgencia' con campos de nombre, género y tipo de sangre, y el botón de registro de urgencia.</t>
+  </si>
+  <si>
+    <t>// Backend: endpoint GET /api/enfermero/paciente/:doc
+if (triExiste.rows.length &gt; 0) {
+  return res.json({
+    encontrado: true,
+    estado: 'YA_REGISTRADO',
+    citId: r.cit_id, ...
+  })
+}
+// Frontend:
+if (data.estado === 'YA_REGISTRADO') {
+  showError('Este paciente ya tiene una urgencia activa.')
+  return
+}</t>
+  </si>
+  <si>
+    <t>El sistema debe mostrar un toast de error indicando que el paciente ya tiene una urgencia activa y no debe permitir abrir un nuevo proceso.</t>
+  </si>
+  <si>
+    <t>El sistema muestra el mensaje de error 'Este paciente ya tiene una urgencia activa. Debe ser atendido primero.' y bloquea el formulario.</t>
+  </si>
+  <si>
+    <t>if (data.success) {
+  onSubmit({ id: data.triId, documento,
+    nombre: paciente.nombre,
+    triage: formData.triage,
+    fechaHora: new Date().toISOString() })
+  success('Triage registrado exitosamente')
+  setDocumento('')
+  setPaciente(null)
+  setFormData({ presionArterial: '', ... })
+}</t>
+  </si>
+  <si>
+    <t>El sistema debe mostrar el toast 'Triage registrado exitosamente', limpiar el formulario y agregar al paciente en el reporte diario.</t>
+  </si>
+  <si>
+    <t>El sistema muestra el toast de confirmación verde, resetea el formulario y el paciente aparece en el listado del reporte diario.</t>
+  </si>
+  <si>
+    <t>if (!formData.urgNombre?.trim()) {
+  errsUrg.urgNombre = 'El nombre es obligatorio'
+} else if (!/^[a-zA-ZáéíóúÁÉÍÓÚñÑüÜ\s]+$/
+    .test(formData.urgNombre.trim())) {
+  errsUrg.urgNombre = 'Solo se permiten letras'
+}</t>
+  </si>
+  <si>
+    <t>El sistema debe mostrar 'Solo se permiten letras' bajo el campo nombre y bloquear el botón 'Registrar como Urgencia y Continuar'.</t>
+  </si>
+  <si>
+    <t>El campo nombre muestra el mensaje de validación 'Solo se permiten letras' y el botón de registro queda bloqueado hasta corregir el dato.</t>
+  </si>
+  <si>
+    <t>if (!formData.urgGenero ||
+    formData.urgGenero === 'D' ||
+    formData.urgGenero === 'DESCONOCIDO') {
+  errsUrg.urgGenero = 'Seleccione un género'
+}
+if (!formData.urgTipoSangre ||
+    formData.urgTipoSangre === 'DESCONOCIDO') {
+  errsUrg.urgTipoSangre = 'Seleccione el tipo de sangre'
+}</t>
+  </si>
+  <si>
+    <t>El sistema debe mostrar 'Seleccione un género' y/o 'Seleccione el tipo de sangre' y bloquear el registro de la urgencia.</t>
+  </si>
+  <si>
+    <t>El sistema muestra los mensajes de error bajo los campos correspondientes y bloquea el registro hasta seleccionar valores válidos.</t>
+  </si>
+  <si>
+    <t>// En VistaReporte — tbody:
+{todos.length === 0 ? (
+  &lt;tr&gt;
+    &lt;td colSpan='4' className='no-results'&gt;
+      No hay pacientes registrados hoy.
+    &lt;/td&gt;
+  &lt;/tr&gt;
+) : todos.map(pac =&gt; (...))}</t>
+  </si>
+  <si>
+    <t>La tabla del reporte debe mostrar el mensaje 'No hay pacientes registrados hoy.' cuando no existen triages para la fecha actual.</t>
+  </si>
+  <si>
+    <t>La tabla muestra el mensaje 'No hay pacientes registrados hoy.' centrado cuando no hay registros de triage en el turno actual.</t>
+  </si>
+  <si>
+    <t>const stats = { I:0, II:0, III:0, IV:0, V:0,
+  total: todos.length }
+todos.forEach(p =&gt; {
+  if (stats[p.nivel] !== undefined)
+    stats[p.nivel]++
+})</t>
+  </si>
+  <si>
+    <t>Las tarjetas de resumen deben mostrar el conteo correcto de pacientes por cada nivel de triage y el total general del día.</t>
+  </si>
+  <si>
+    <t>Las tarjetas de resumen muestran los conteos correctos por nivel (I a V) y el total de pacientes atendidos durante el turno.</t>
+  </si>
+  <si>
+    <t>// Sección print-only con encabezado CMQ:
+&lt;div className='print-only'&gt;
+  &lt;div&gt;HOSPITAL CMQ&lt;/div&gt;
+  &lt;div&gt;Reporte de Gestión Diario — Área de Triage&lt;/div&gt;
+  &lt;span&gt;Fecha: {hoy}&lt;/span&gt;
+  &lt;span&gt;Enfermero: {usuario.nombre || '—'}&lt;/span&gt;
+  // Tabla + firma al pie
+  &lt;button onClick={() =&gt; window.print()}&gt;
+    Imprimir PDF
+  &lt;/button&gt;
+&lt;/div&gt;</t>
+  </si>
+  <si>
+    <t>El documento generado debe incluir encabezado institucional 'HOSPITAL CMQ', fecha, nombre del enfermero, tabla de pacientes y espacio de firma.</t>
+  </si>
+  <si>
+    <t>Al imprimir, el documento muestra el encabezado institucional, la fecha, el nombre del enfermero, la tabla de atenciones y la línea de firma.</t>
   </si>
 </sst>
 </file>
@@ -717,7 +890,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -772,6 +945,18 @@
         <bgColor rgb="FF008080"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor rgb="FFF1F5F9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor rgb="FFFFFF99"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -800,7 +985,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -830,11 +1015,14 @@
     <xf numFmtId="0" fontId="11" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -842,45 +1030,28 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1637,6 +1808,540 @@
         <a:xfrm>
           <a:off x="16399565" y="14116349"/>
           <a:ext cx="5932419" cy="1419994"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>1925483</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>61450</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>4452619</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>2488790</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Imagen 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5C73A5E0-AD48-48CB-A89B-C1F05422268D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="18251128" y="1013950"/>
+          <a:ext cx="2527136" cy="2427340"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>1177823</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>686209</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>5131250</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>1819842</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Imagen 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5112595D-3E41-46AB-AA3F-86F54D4B81AD}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="17503468" y="4168467"/>
+          <a:ext cx="3953427" cy="1133633"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>215080</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>409677</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>5950565</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>2162376</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Imagen 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8337BC96-0F4A-46A1-828C-388EE4AB17E8}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="16540725" y="6421693"/>
+          <a:ext cx="5735485" cy="1752699"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>184355</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>758199</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>5981291</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>1781346</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Imagen 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CF36B0B5-5486-4EA8-A85F-589CB44C7328}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="16510000" y="9299973"/>
+          <a:ext cx="5796936" cy="1023147"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>686208</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>81934</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>5312907</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>2427339</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Imagen 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0FCBDB33-354F-4793-822B-67E9B815B2C6}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="17011853" y="11153466"/>
+          <a:ext cx="4626699" cy="2345405"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>860322</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>706693</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>5251151</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>1792338</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="Imagen 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B67BB6A6-1674-4D82-96AD-0622B47486ED}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="17185967" y="14307983"/>
+          <a:ext cx="4390829" cy="1085645"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>1116371</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>686210</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>5104086</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>1689920</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="8" name="Imagen 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C1CCEE55-14BF-4AAB-8DA8-7D34ECCDEC06}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="17442016" y="16817258"/>
+          <a:ext cx="3987715" cy="1003710"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>993467</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>614517</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>5120968</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>2055351</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="9" name="Imagen 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{13CA9B5C-C968-4EB3-99A0-06A79E8AD3A3}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="17319112" y="19275323"/>
+          <a:ext cx="4127501" cy="1440834"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>583790</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>542821</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>5575405</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>1945966</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="10" name="Imagen 9">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CAB8C45D-0BB2-40D3-B038-2355DB27E48B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="16909435" y="21733386"/>
+          <a:ext cx="4991615" cy="1403145"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>130736</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>803088</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>5919839</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>1592027</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="11" name="Imagen 10">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C9DD3A13-D669-4375-ABDE-0606180A76E2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="16456381" y="27053169"/>
+          <a:ext cx="5789103" cy="788939"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>1802578</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>92177</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>4557661</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>2422603</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="12" name="Imagen 11">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6C276BB8-A661-4031-BF30-A28FDA1BF30E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="18128223" y="28872016"/>
+          <a:ext cx="2755083" cy="2330426"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>159653</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>503060</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>5959710</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>2027903</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="13" name="Imagen 12">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DE240D5F-C112-34AB-829D-B86ABCA94619}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12"/>
+        <a:srcRect t="53274" r="40209"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="16485298" y="24223383"/>
+          <a:ext cx="5800057" cy="1524843"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1846,30 +2551,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
-      <c r="I1" s="13"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
+      <c r="H1" s="14"/>
+      <c r="I1" s="14"/>
     </row>
     <row r="2" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="14"/>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14"/>
-      <c r="F2" s="14"/>
-      <c r="G2" s="14"/>
-      <c r="H2" s="14"/>
-      <c r="I2" s="14"/>
+      <c r="B2" s="15"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="15"/>
+      <c r="G2" s="15"/>
+      <c r="H2" s="15"/>
+      <c r="I2" s="15"/>
     </row>
     <row r="3" spans="1:10" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -1974,7 +2679,7 @@
         <v>28</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>145</v>
+        <v>133</v>
       </c>
       <c r="E6" s="9" t="s">
         <v>29</v>
@@ -2078,7 +2783,7 @@
       <c r="H9" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="I9" s="19" t="s">
+      <c r="I9" s="12" t="s">
         <v>19</v>
       </c>
       <c r="J9" s="7"/>
@@ -2129,16 +2834,16 @@
       <c r="E11" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="F11" s="16" t="s">
-        <v>146</v>
-      </c>
-      <c r="G11" s="15" t="s">
-        <v>147</v>
-      </c>
-      <c r="H11" s="15" t="s">
-        <v>148</v>
-      </c>
-      <c r="I11" s="17" t="s">
+      <c r="F11" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="H11" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="I11" s="6" t="s">
         <v>19</v>
       </c>
       <c r="J11" s="7"/>
@@ -2159,16 +2864,16 @@
       <c r="E12" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="F12" s="16" t="s">
-        <v>149</v>
-      </c>
-      <c r="G12" s="15" t="s">
-        <v>150</v>
-      </c>
-      <c r="H12" s="15" t="s">
-        <v>151</v>
-      </c>
-      <c r="I12" s="17" t="s">
+      <c r="F12" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="I12" s="6" t="s">
         <v>19</v>
       </c>
       <c r="J12" s="7"/>
@@ -2189,16 +2894,16 @@
       <c r="E13" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="F13" s="16" t="s">
-        <v>152</v>
-      </c>
-      <c r="G13" s="15" t="s">
-        <v>153</v>
-      </c>
-      <c r="H13" s="15" t="s">
-        <v>154</v>
-      </c>
-      <c r="I13" s="17" t="s">
+      <c r="F13" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="G13" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="H13" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="I13" s="6" t="s">
         <v>19</v>
       </c>
       <c r="J13" s="7"/>
@@ -2217,18 +2922,18 @@
         <v>75</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>167</v>
-      </c>
-      <c r="F14" s="16" t="s">
         <v>155</v>
       </c>
-      <c r="G14" s="15" t="s">
-        <v>156</v>
-      </c>
-      <c r="H14" s="15" t="s">
-        <v>157</v>
-      </c>
-      <c r="I14" s="17" t="s">
+      <c r="F14" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="G14" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="H14" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="I14" s="6" t="s">
         <v>19</v>
       </c>
       <c r="J14" s="7"/>
@@ -2247,18 +2952,18 @@
         <v>78</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>166</v>
-      </c>
-      <c r="F15" s="16" t="s">
-        <v>165</v>
-      </c>
-      <c r="G15" s="15" t="s">
-        <v>164</v>
-      </c>
-      <c r="H15" s="15" t="s">
-        <v>158</v>
-      </c>
-      <c r="I15" s="17" t="s">
+        <v>154</v>
+      </c>
+      <c r="F15" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="G15" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="H15" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="I15" s="6" t="s">
         <v>19</v>
       </c>
       <c r="J15" s="7"/>
@@ -2279,35 +2984,35 @@
       <c r="E16" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="F16" s="16" t="s">
-        <v>159</v>
-      </c>
-      <c r="G16" s="15" t="s">
-        <v>160</v>
-      </c>
-      <c r="H16" s="15" t="s">
-        <v>161</v>
-      </c>
-      <c r="I16" s="17" t="s">
+      <c r="F16" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="G16" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="H16" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="I16" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="J16" s="18" t="s">
-        <v>168</v>
+      <c r="J16" s="11" t="s">
+        <v>156</v>
       </c>
     </row>
     <row r="17" spans="1:9" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="11" t="s">
-        <v>163</v>
-      </c>
-      <c r="B17" s="12"/>
-      <c r="C17" s="12"/>
-      <c r="D17" s="12"/>
-      <c r="E17" s="12"/>
-      <c r="F17" s="12"/>
-      <c r="G17" s="12"/>
-      <c r="H17" s="12"/>
+      <c r="A17" s="16" t="s">
+        <v>151</v>
+      </c>
+      <c r="B17" s="17"/>
+      <c r="C17" s="17"/>
+      <c r="D17" s="17"/>
+      <c r="E17" s="17"/>
+      <c r="F17" s="17"/>
+      <c r="G17" s="17"/>
+      <c r="H17" s="17"/>
       <c r="I17" s="10" t="s">
-        <v>162</v>
+        <v>150</v>
       </c>
     </row>
   </sheetData>
@@ -2324,7 +3029,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:J19"/>
+  <dimension ref="A1:J18"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -2340,446 +3045,470 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="14" t="s">
         <v>83</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
-      <c r="I1" s="13"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
+      <c r="H1" s="14"/>
+      <c r="I1" s="14"/>
     </row>
     <row r="2" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="20" t="s">
+      <c r="A2" s="18" t="s">
         <v>84</v>
       </c>
-      <c r="B2" s="14"/>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14"/>
-      <c r="F2" s="14"/>
-      <c r="G2" s="14"/>
-      <c r="H2" s="14"/>
-      <c r="I2" s="14"/>
+      <c r="B2" s="15"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="15"/>
+      <c r="G2" s="15"/>
+      <c r="H2" s="15"/>
+      <c r="I2" s="15"/>
     </row>
     <row r="3" spans="1:10" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="22" t="s">
+      <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="22" t="s">
+      <c r="B3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="22" t="s">
+      <c r="C3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="22" t="s">
+      <c r="D3" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="22" t="s">
+      <c r="E3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F3" s="22" t="s">
+      <c r="F3" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="G3" s="22" t="s">
+      <c r="G3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="H3" s="22" t="s">
+      <c r="H3" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="I3" s="22" t="s">
+      <c r="I3" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="J3" s="22" t="s">
+      <c r="J3" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="200.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="23">
+      <c r="A4" s="2">
         <v>1</v>
       </c>
-      <c r="B4" s="24" t="s">
+      <c r="B4" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="C4" s="24" t="s">
+      <c r="C4" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="D4" s="24" t="s">
+      <c r="D4" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="E4" s="25" t="s">
+      <c r="E4" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="F4" s="26"/>
-      <c r="G4" s="24"/>
-      <c r="H4" s="24"/>
-      <c r="I4" s="27" t="s">
+      <c r="F4" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="I4" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="J4" s="28"/>
+      <c r="J4" s="7"/>
     </row>
     <row r="5" spans="1:10" ht="200.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="23">
+      <c r="A5" s="2">
         <v>2</v>
       </c>
-      <c r="B5" s="24" t="s">
+      <c r="B5" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C5" s="24" t="s">
+      <c r="C5" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="D5" s="24" t="s">
+      <c r="D5" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="E5" s="25" t="s">
+      <c r="E5" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="F5" s="26"/>
-      <c r="G5" s="24"/>
-      <c r="H5" s="24"/>
-      <c r="I5" s="27" t="s">
+      <c r="F5" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="I5" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="J5" s="28"/>
+      <c r="J5" s="7"/>
     </row>
     <row r="6" spans="1:10" ht="200.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="23">
+      <c r="A6" s="2">
         <v>3</v>
       </c>
-      <c r="B6" s="24" t="s">
+      <c r="B6" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="C6" s="24" t="s">
+      <c r="C6" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="D6" s="24" t="s">
+      <c r="D6" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="E6" s="25" t="s">
+      <c r="E6" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="F6" s="26"/>
-      <c r="G6" s="24"/>
-      <c r="H6" s="24"/>
-      <c r="I6" s="27" t="s">
+      <c r="F6" s="5" t="s">
+        <v>165</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="I6" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="J6" s="28"/>
+      <c r="J6" s="7"/>
     </row>
     <row r="7" spans="1:10" ht="200.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="23">
+      <c r="A7" s="2">
         <v>4</v>
       </c>
-      <c r="B7" s="24" t="s">
+      <c r="B7" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="C7" s="24" t="s">
+      <c r="C7" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="D7" s="24" t="s">
+      <c r="D7" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="E7" s="25" t="s">
+      <c r="E7" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="F7" s="26"/>
-      <c r="G7" s="24"/>
-      <c r="H7" s="24"/>
-      <c r="I7" s="27" t="s">
+      <c r="F7" s="5" t="s">
+        <v>168</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="I7" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="J7" s="28"/>
+      <c r="J7" s="7"/>
     </row>
     <row r="8" spans="1:10" ht="200.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="23">
+      <c r="A8" s="2">
         <v>5</v>
       </c>
-      <c r="B8" s="24" t="s">
+      <c r="B8" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="C8" s="24" t="s">
+      <c r="C8" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="D8" s="24" t="s">
+      <c r="D8" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="E8" s="25" t="s">
+      <c r="E8" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="F8" s="26"/>
-      <c r="G8" s="24"/>
-      <c r="H8" s="24"/>
-      <c r="I8" s="27" t="s">
+      <c r="F8" s="5" t="s">
+        <v>171</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="I8" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="J8" s="28"/>
+      <c r="J8" s="7"/>
     </row>
     <row r="9" spans="1:10" ht="200.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="23">
+      <c r="A9" s="2">
         <v>6</v>
       </c>
-      <c r="B9" s="24" t="s">
+      <c r="B9" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="C9" s="24" t="s">
+      <c r="C9" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="D9" s="24" t="s">
+      <c r="D9" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="E9" s="25" t="s">
+      <c r="E9" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="F9" s="26"/>
-      <c r="G9" s="24"/>
-      <c r="H9" s="24"/>
-      <c r="I9" s="27" t="s">
+      <c r="F9" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="H9" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="I9" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="J9" s="28"/>
+      <c r="J9" s="7"/>
     </row>
     <row r="10" spans="1:10" ht="200.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="23">
+      <c r="A10" s="2">
         <v>7</v>
       </c>
-      <c r="B10" s="24" t="s">
+      <c r="B10" s="3" t="s">
         <v>109</v>
       </c>
-      <c r="C10" s="24" t="s">
+      <c r="C10" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="D10" s="24" t="s">
+      <c r="D10" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="E10" s="25" t="s">
+      <c r="E10" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="F10" s="26"/>
-      <c r="G10" s="24"/>
-      <c r="H10" s="24"/>
-      <c r="I10" s="27" t="s">
+      <c r="F10" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="I10" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="J10" s="28"/>
+      <c r="J10" s="7"/>
     </row>
     <row r="11" spans="1:10" ht="200.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="23">
+      <c r="A11" s="2">
         <v>8</v>
       </c>
-      <c r="B11" s="24" t="s">
+      <c r="B11" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="C11" s="24" t="s">
+      <c r="C11" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="D11" s="24" t="s">
+      <c r="D11" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="E11" s="25" t="s">
+      <c r="E11" s="4" t="s">
         <v>116</v>
       </c>
-      <c r="F11" s="26"/>
-      <c r="G11" s="24"/>
-      <c r="H11" s="24"/>
-      <c r="I11" s="27" t="s">
+      <c r="F11" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="H11" s="3" t="s">
+        <v>182</v>
+      </c>
+      <c r="I11" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="J11" s="28"/>
+      <c r="J11" s="7"/>
     </row>
     <row r="12" spans="1:10" ht="200.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="23">
+      <c r="A12" s="2">
         <v>9</v>
       </c>
-      <c r="B12" s="24" t="s">
+      <c r="B12" s="3" t="s">
         <v>117</v>
       </c>
-      <c r="C12" s="24" t="s">
+      <c r="C12" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="D12" s="24" t="s">
+      <c r="D12" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="E12" s="25" t="s">
+      <c r="E12" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="F12" s="26"/>
-      <c r="G12" s="24"/>
-      <c r="H12" s="24"/>
-      <c r="I12" s="27" t="s">
+      <c r="F12" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>184</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="I12" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="J12" s="28"/>
+      <c r="J12" s="7"/>
     </row>
     <row r="13" spans="1:10" ht="200.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="23">
+      <c r="A13" s="2">
         <v>10</v>
       </c>
-      <c r="B13" s="24" t="s">
+      <c r="B13" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="C13" s="24" t="s">
+      <c r="C13" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="D13" s="24" t="s">
+      <c r="D13" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="E13" s="25" t="s">
+      <c r="E13" s="4" t="s">
         <v>124</v>
       </c>
-      <c r="F13" s="26"/>
-      <c r="G13" s="24"/>
-      <c r="H13" s="24"/>
-      <c r="I13" s="27" t="s">
+      <c r="F13" s="5" t="s">
+        <v>186</v>
+      </c>
+      <c r="G13" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="H13" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="I13" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="J13" s="28"/>
+      <c r="J13" s="7"/>
     </row>
     <row r="14" spans="1:10" ht="200.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="23">
+      <c r="A14" s="2">
         <v>11</v>
       </c>
-      <c r="B14" s="24" t="s">
+      <c r="B14" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="C14" s="24" t="s">
+      <c r="C14" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="D14" s="24" t="s">
+      <c r="D14" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="E14" s="25" t="s">
+      <c r="E14" s="4" t="s">
         <v>128</v>
       </c>
-      <c r="F14" s="26"/>
-      <c r="G14" s="24"/>
-      <c r="H14" s="24"/>
-      <c r="I14" s="27" t="s">
+      <c r="F14" s="5" t="s">
+        <v>189</v>
+      </c>
+      <c r="G14" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="H14" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="I14" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="J14" s="28"/>
+      <c r="J14" s="7"/>
     </row>
     <row r="15" spans="1:10" ht="200.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="23">
+      <c r="A15" s="2">
         <v>12</v>
       </c>
-      <c r="B15" s="24" t="s">
+      <c r="B15" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="C15" s="24" t="s">
+      <c r="C15" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="D15" s="24" t="s">
+      <c r="D15" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="E15" s="25" t="s">
+      <c r="E15" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="F15" s="26"/>
-      <c r="G15" s="24"/>
-      <c r="H15" s="24"/>
-      <c r="I15" s="27" t="s">
+      <c r="F15" s="5" t="s">
+        <v>192</v>
+      </c>
+      <c r="G15" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="H15" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="I15" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="J15" s="28"/>
+      <c r="J15" s="7"/>
     </row>
-    <row r="16" spans="1:10" ht="200.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="23">
-        <v>13</v>
-      </c>
-      <c r="B16" s="24" t="s">
-        <v>133</v>
-      </c>
-      <c r="C16" s="24" t="s">
-        <v>134</v>
-      </c>
-      <c r="D16" s="24" t="s">
-        <v>135</v>
-      </c>
-      <c r="E16" s="25" t="s">
-        <v>136</v>
-      </c>
-      <c r="F16" s="26"/>
-      <c r="G16" s="24"/>
-      <c r="H16" s="24"/>
-      <c r="I16" s="27" t="s">
-        <v>19</v>
-      </c>
-      <c r="J16" s="28"/>
+    <row r="16" spans="1:10" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="17" t="s">
+        <v>158</v>
+      </c>
+      <c r="B16" s="17"/>
+      <c r="C16" s="17"/>
+      <c r="D16" s="17"/>
+      <c r="E16" s="17"/>
+      <c r="F16" s="17"/>
+      <c r="G16" s="17"/>
+      <c r="H16" s="17"/>
+      <c r="I16" s="13" t="s">
+        <v>157</v>
+      </c>
     </row>
-    <row r="17" spans="1:10" ht="200.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="23">
-        <v>14</v>
-      </c>
-      <c r="B17" s="24" t="s">
-        <v>137</v>
-      </c>
-      <c r="C17" s="24" t="s">
-        <v>138</v>
-      </c>
-      <c r="D17" s="24" t="s">
-        <v>139</v>
-      </c>
-      <c r="E17" s="25" t="s">
-        <v>140</v>
-      </c>
-      <c r="F17" s="26"/>
-      <c r="G17" s="24"/>
-      <c r="H17" s="24"/>
-      <c r="I17" s="27" t="s">
-        <v>19</v>
-      </c>
-      <c r="J17" s="28"/>
+    <row r="17" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="19"/>
+      <c r="B17" s="20"/>
+      <c r="C17" s="20"/>
+      <c r="D17" s="20"/>
+      <c r="E17" s="21"/>
+      <c r="F17" s="22"/>
+      <c r="G17" s="20"/>
+      <c r="H17" s="20"/>
+      <c r="I17" s="23"/>
+      <c r="J17" s="7"/>
     </row>
-    <row r="18" spans="1:10" ht="200.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="23">
-        <v>15</v>
-      </c>
-      <c r="B18" s="24" t="s">
-        <v>141</v>
-      </c>
-      <c r="C18" s="24" t="s">
-        <v>142</v>
-      </c>
-      <c r="D18" s="24" t="s">
-        <v>143</v>
-      </c>
-      <c r="E18" s="25" t="s">
-        <v>144</v>
-      </c>
-      <c r="F18" s="26"/>
-      <c r="G18" s="24"/>
-      <c r="H18" s="24"/>
-      <c r="I18" s="27" t="s">
-        <v>19</v>
-      </c>
-      <c r="J18" s="28"/>
-    </row>
-    <row r="19" spans="1:10" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="12" t="s">
-        <v>169</v>
-      </c>
-      <c r="B19" s="12"/>
-      <c r="C19" s="12"/>
-      <c r="D19" s="12"/>
-      <c r="E19" s="12"/>
-      <c r="F19" s="12"/>
-      <c r="G19" s="12"/>
-      <c r="H19" s="12"/>
-      <c r="I19" s="29" t="s">
-        <v>170</v>
-      </c>
-      <c r="J19" s="21"/>
+    <row r="18" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="19"/>
+      <c r="B18" s="20"/>
+      <c r="C18" s="20"/>
+      <c r="D18" s="20"/>
+      <c r="E18" s="21"/>
+      <c r="F18" s="22"/>
+      <c r="G18" s="20"/>
+      <c r="H18" s="20"/>
+      <c r="I18" s="23"/>
+      <c r="J18" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A2:I2"/>
-    <mergeCell ref="A19:H19"/>
+    <mergeCell ref="A16:H16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix; codigo prueba(PU-ENF-005) registrar como urgncia
</commit_message>
<xml_diff>
--- a/docs/Pruebas_Unitarias_CMQ_V4.xlsx
+++ b/docs/Pruebas_Unitarias_CMQ_V4.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\crist\PROYECTOS_2026_I\Proyecto_IngSoft_SP4\ultima_entrega_cmq\cmq-medical-data-integration\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8299BE4A-0B45-4185-85B4-C3076445E51A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6C29131-92C5-4B73-95D0-F7A0E5929132}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -658,16 +658,6 @@
     <t>El formulario muestra el banner de alertas clínicas con los mensajes de taquicardia, fiebre o saturación crítica en tiempo real al escribir.</t>
   </si>
   <si>
-    <t>if (!data.encontrado) {
-  setNoEncontrado(true)
-}
-// En el render se muestra el panel
-// 'Registrar como Urgencia' con campos:
-// urgNombre, urgGenero, urgTipoSangre
-// y el botón:
-// '🚨 Registrar como Urgencia y Continuar'</t>
-  </si>
-  <si>
     <t>El sistema debe informar que el paciente no fue encontrado y mostrar un formulario para registrarlo como urgencia antes de continuar con el triage.</t>
   </si>
   <si>
@@ -791,6 +781,27 @@
   </si>
   <si>
     <t>Al imprimir, el documento muestra el encabezado institucional, la fecha, el nombre del enfermero, la tabla de atenciones y la línea de firma.</t>
+  </si>
+  <si>
+    <t>if (data.encontrado) {
+        if (data.estado === 'YA_REGISTRADO') {
+          showError('Este paciente ya tiene una urgencia activa. Debe ser atendido primero.')
+          return
+        }
+        setPaciente(data)
+      } else {
+        setNoEncontrado(true)
+      }// En el render se muestra el panel
+// 'Registrar como Urgencia' con campos:
+// urgNombre, urgGenero, urgTipoSangre
+// y el botón:
+color: 'white', border: 'none', borderRadius: '6px',
+padding: '10px 20px', fontWeight: 700, cursor: 'pointer',
+      }}
+    &gt;
+      🚨 Registrar como Urgencia y Continuar
+    &lt;/button&gt;
+  &lt;/div&gt;</t>
   </si>
 </sst>
 </file>
@@ -3239,13 +3250,13 @@
         <v>104</v>
       </c>
       <c r="F8" s="5" t="s">
+        <v>194</v>
+      </c>
+      <c r="G8" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="G8" s="3" t="s">
+      <c r="H8" s="3" t="s">
         <v>172</v>
-      </c>
-      <c r="H8" s="3" t="s">
-        <v>173</v>
       </c>
       <c r="I8" s="6" t="s">
         <v>19</v>
@@ -3269,13 +3280,13 @@
         <v>108</v>
       </c>
       <c r="F9" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="G9" s="3" t="s">
         <v>174</v>
       </c>
-      <c r="G9" s="3" t="s">
+      <c r="H9" s="3" t="s">
         <v>175</v>
-      </c>
-      <c r="H9" s="3" t="s">
-        <v>176</v>
       </c>
       <c r="I9" s="6" t="s">
         <v>19</v>
@@ -3299,13 +3310,13 @@
         <v>112</v>
       </c>
       <c r="F10" s="5" t="s">
+        <v>176</v>
+      </c>
+      <c r="G10" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="G10" s="3" t="s">
+      <c r="H10" s="3" t="s">
         <v>178</v>
-      </c>
-      <c r="H10" s="3" t="s">
-        <v>179</v>
       </c>
       <c r="I10" s="6" t="s">
         <v>19</v>
@@ -3329,13 +3340,13 @@
         <v>116</v>
       </c>
       <c r="F11" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="G11" s="3" t="s">
         <v>180</v>
       </c>
-      <c r="G11" s="3" t="s">
+      <c r="H11" s="3" t="s">
         <v>181</v>
-      </c>
-      <c r="H11" s="3" t="s">
-        <v>182</v>
       </c>
       <c r="I11" s="6" t="s">
         <v>19</v>
@@ -3359,13 +3370,13 @@
         <v>120</v>
       </c>
       <c r="F12" s="5" t="s">
+        <v>182</v>
+      </c>
+      <c r="G12" s="3" t="s">
         <v>183</v>
       </c>
-      <c r="G12" s="3" t="s">
+      <c r="H12" s="3" t="s">
         <v>184</v>
-      </c>
-      <c r="H12" s="3" t="s">
-        <v>185</v>
       </c>
       <c r="I12" s="6" t="s">
         <v>19</v>
@@ -3389,13 +3400,13 @@
         <v>124</v>
       </c>
       <c r="F13" s="5" t="s">
+        <v>185</v>
+      </c>
+      <c r="G13" s="3" t="s">
         <v>186</v>
       </c>
-      <c r="G13" s="3" t="s">
+      <c r="H13" s="3" t="s">
         <v>187</v>
-      </c>
-      <c r="H13" s="3" t="s">
-        <v>188</v>
       </c>
       <c r="I13" s="6" t="s">
         <v>19</v>
@@ -3419,13 +3430,13 @@
         <v>128</v>
       </c>
       <c r="F14" s="5" t="s">
+        <v>188</v>
+      </c>
+      <c r="G14" s="3" t="s">
         <v>189</v>
       </c>
-      <c r="G14" s="3" t="s">
+      <c r="H14" s="3" t="s">
         <v>190</v>
-      </c>
-      <c r="H14" s="3" t="s">
-        <v>191</v>
       </c>
       <c r="I14" s="6" t="s">
         <v>19</v>
@@ -3449,13 +3460,13 @@
         <v>132</v>
       </c>
       <c r="F15" s="5" t="s">
+        <v>191</v>
+      </c>
+      <c r="G15" s="3" t="s">
         <v>192</v>
       </c>
-      <c r="G15" s="3" t="s">
+      <c r="H15" s="3" t="s">
         <v>193</v>
-      </c>
-      <c r="H15" s="3" t="s">
-        <v>194</v>
       </c>
       <c r="I15" s="6" t="s">
         <v>19</v>

</xml_diff>